<commit_message>
Removing flights with fog and updating models
</commit_message>
<xml_diff>
--- a/Jones_honours/01_raw_data/DFO_data/DFO_flight_logs/Subarea visibily 2021_2022.xlsx
+++ b/Jones_honours/01_raw_data/DFO_data/DFO_flight_logs/Subarea visibily 2021_2022.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alecjones/Documents/GitHub/Alec_Jones_Honours/Jones_honours/01_raw_data/DFO_data/DFO_flight_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B822E275-36B9-1341-8ED6-51A4EF78606E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C739738-6B6B-9142-A20C-2CBAEA66F242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{0C36C268-8746-4F89-B6F9-4FA6A4150BF7}"/>
+    <workbookView xWindow="19300" yWindow="580" windowWidth="18960" windowHeight="11380" activeTab="1" xr2:uid="{0C36C268-8746-4F89-B6F9-4FA6A4150BF7}"/>
   </bookViews>
   <sheets>
     <sheet name="2021 flight visibility" sheetId="2" r:id="rId1"/>
@@ -493,6 +493,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>177800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>596900</xdr:colOff>
+      <xdr:row>118</xdr:row>
+      <xdr:rowOff>140541</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{932AEB56-66B0-E99D-210C-220CA81B592E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13157200" y="6083300"/>
+          <a:ext cx="7772400" cy="9868741"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -913,7 +962,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>61</v>
       </c>
@@ -955,7 +1004,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>92</v>
       </c>
@@ -969,7 +1018,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>92</v>
       </c>
@@ -998,7 +1047,7 @@
       </c>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>92</v>
       </c>
@@ -1012,7 +1061,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>92</v>
       </c>
@@ -1026,7 +1075,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>92</v>
       </c>
@@ -1040,7 +1089,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>92</v>
       </c>
@@ -1054,7 +1103,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>92</v>
       </c>
@@ -1068,7 +1117,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>92</v>
       </c>
@@ -1082,7 +1131,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>92</v>
       </c>
@@ -1096,7 +1145,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>92</v>
       </c>
@@ -1110,7 +1159,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>92</v>
       </c>
@@ -1124,7 +1173,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>92</v>
       </c>
@@ -1194,7 +1243,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>92</v>
       </c>
@@ -1222,7 +1271,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>92</v>
       </c>
@@ -1236,7 +1285,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>92</v>
       </c>
@@ -1306,7 +1355,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>92</v>
       </c>
@@ -1334,7 +1383,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>92</v>
       </c>
@@ -1362,7 +1411,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>92</v>
       </c>
@@ -1376,7 +1425,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>92</v>
       </c>
@@ -1404,7 +1453,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>92</v>
       </c>
@@ -1418,7 +1467,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>92</v>
       </c>
@@ -1432,7 +1481,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>92</v>
       </c>
@@ -1446,7 +1495,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>92</v>
       </c>
@@ -1460,7 +1509,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>92</v>
       </c>
@@ -1474,7 +1523,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>76</v>
       </c>
@@ -1544,7 +1593,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>76</v>
       </c>
@@ -1572,7 +1621,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>76</v>
       </c>
@@ -1600,7 +1649,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>76</v>
       </c>
@@ -1614,7 +1663,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>76</v>
       </c>
@@ -1642,7 +1691,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>76</v>
       </c>
@@ -1656,7 +1705,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>76</v>
       </c>
@@ -1670,7 +1719,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>76</v>
       </c>
@@ -1684,7 +1733,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>76</v>
       </c>
@@ -1698,7 +1747,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>76</v>
       </c>
@@ -1712,7 +1761,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>76</v>
       </c>
@@ -1726,7 +1775,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
         <v>76</v>
       </c>
@@ -1740,7 +1789,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
         <v>76</v>
       </c>
@@ -1782,7 +1831,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
         <v>76</v>
       </c>
@@ -1894,7 +1943,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="79" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
         <v>65</v>
       </c>
@@ -1936,7 +1985,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="82" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:36" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>65</v>
       </c>
@@ -1964,7 +2013,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="84" spans="1:36" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:36" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>65</v>
       </c>
@@ -2010,7 +2059,7 @@
       <c r="AI84"/>
       <c r="AJ84"/>
     </row>
-    <row r="85" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:36" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>65</v>
       </c>
@@ -2074,15 +2123,17 @@
   <autoFilter ref="A1:D88" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="2">
       <filters>
-        <filter val="24D"/>
-        <filter val="24E"/>
-        <filter val="24I"/>
-        <filter val="24J"/>
-        <filter val="24K"/>
-        <filter val="24L"/>
-        <filter val="24M"/>
-        <filter val="24N"/>
-        <filter val="24O"/>
+        <filter val="23A"/>
+        <filter val="23B"/>
+        <filter val="23C"/>
+        <filter val="23D"/>
+        <filter val="23F"/>
+        <filter val="23I"/>
+        <filter val="23J"/>
+        <filter val="23K"/>
+        <filter val="23M"/>
+        <filter val="23O"/>
+        <filter val="23P"/>
         <filter val="all areas"/>
       </filters>
     </filterColumn>
@@ -2094,6 +2145,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D648FCB-8485-434D-BD77-AE02B41E8302}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2152,7 +2204,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>44716</v>
       </c>
@@ -2166,7 +2218,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>44716</v>
       </c>
@@ -2177,7 +2229,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>44716</v>
       </c>
@@ -2188,7 +2240,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>44716</v>
       </c>
@@ -2199,7 +2251,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>44716</v>
       </c>
@@ -2213,7 +2265,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>44716</v>
       </c>
@@ -2227,7 +2279,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>44716</v>
       </c>
@@ -2252,7 +2304,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>44740</v>
       </c>
@@ -2263,7 +2315,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>44740</v>
       </c>
@@ -2274,7 +2326,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>44740</v>
       </c>
@@ -2296,7 +2348,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>44760</v>
       </c>
@@ -2307,7 +2359,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>44760</v>
       </c>
@@ -2318,7 +2370,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>44760</v>
       </c>
@@ -2329,7 +2381,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>44765</v>
       </c>
@@ -2395,7 +2447,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>44773</v>
       </c>
@@ -2406,7 +2458,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>44773</v>
       </c>
@@ -2417,7 +2469,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>44773</v>
       </c>
@@ -2428,7 +2480,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>44773</v>
       </c>
@@ -2439,7 +2491,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>44773</v>
       </c>
@@ -2450,7 +2502,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>44783</v>
       </c>
@@ -2461,7 +2513,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>44783</v>
       </c>
@@ -2472,7 +2524,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>44784</v>
       </c>
@@ -2483,7 +2535,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>44784</v>
       </c>
@@ -2494,7 +2546,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>44784</v>
       </c>
@@ -2505,7 +2557,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>44784</v>
       </c>
@@ -2516,7 +2568,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4">
         <v>44787</v>
       </c>
@@ -2549,7 +2601,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>44790</v>
       </c>
@@ -2615,7 +2667,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>44800</v>
       </c>
@@ -2626,7 +2678,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>44809</v>
       </c>
@@ -2637,7 +2689,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>44809</v>
       </c>
@@ -2648,7 +2700,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>44809</v>
       </c>
@@ -2659,7 +2711,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>44809</v>
       </c>
@@ -2670,7 +2722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>44834</v>
       </c>
@@ -2681,7 +2733,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>44834</v>
       </c>
@@ -2692,7 +2744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>44834</v>
       </c>
@@ -2704,9 +2756,25 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C53" xr:uid="{2D28979A-71F1-4F82-BBCC-681E4CA93179}"/>
+  <autoFilter ref="A1:C53" xr:uid="{2D28979A-71F1-4F82-BBCC-681E4CA93179}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="23a"/>
+        <filter val="23b"/>
+        <filter val="23C"/>
+        <filter val="23D"/>
+        <filter val="23F"/>
+        <filter val="23J"/>
+        <filter val="23K"/>
+        <filter val="23O"/>
+        <filter val="23Q"/>
+        <filter val="24D"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Making plots of the evs to look at concurvity
</commit_message>
<xml_diff>
--- a/Jones_honours/01_raw_data/DFO_data/DFO_flight_logs/Subarea visibily 2021_2022.xlsx
+++ b/Jones_honours/01_raw_data/DFO_data/DFO_flight_logs/Subarea visibily 2021_2022.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alecjones/Documents/GitHub/Alec_Jones_Honours/Jones_honours/01_raw_data/DFO_data/DFO_flight_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C739738-6B6B-9142-A20C-2CBAEA66F242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E387BC2A-0146-9443-8CB4-B117A62D36BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19300" yWindow="580" windowWidth="18960" windowHeight="11380" activeTab="1" xr2:uid="{0C36C268-8746-4F89-B6F9-4FA6A4150BF7}"/>
+    <workbookView xWindow="7480" yWindow="1860" windowWidth="18960" windowHeight="10300" activeTab="1" xr2:uid="{0C36C268-8746-4F89-B6F9-4FA6A4150BF7}"/>
   </bookViews>
   <sheets>
     <sheet name="2021 flight visibility" sheetId="2" r:id="rId1"/>

</xml_diff>